<commit_message>
adding sample run data
</commit_message>
<xml_diff>
--- a/Sample_run/1/StudentsSolution.xlsx
+++ b/Sample_run/1/StudentsSolution.xlsx
@@ -55,10 +55,10 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:20:51</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11-12-2025 14:23:03</x:t>
+    <x:t>11-12-2025 14:40:07</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11-12-2025 14:42:12</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -70,7 +70,10 @@
     <x:t>1.5</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:23:07</x:t>
+    <x:t>11-12-2025 14:40:06</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11-12-2025 14:42:13</x:t>
   </x:si>
   <x:si>
     <x:t>3</x:t>
@@ -79,7 +82,7 @@
     <x:t>Control</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:22:59</x:t>
+    <x:t>11-12-2025 14:42:06</x:t>
   </x:si>
   <x:si>
     <x:t>4</x:t>
@@ -91,7 +94,7 @@
     <x:t>0</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:23:11</x:t>
+    <x:t>11-12-2025 14:42:26</x:t>
   </x:si>
   <x:si>
     <x:t>ducnthe180869</x:t>
@@ -106,7 +109,7 @@
     <x:t>dungdvhe181404</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:23:08</x:t>
+    <x:t>11-12-2025 14:42:19</x:t>
   </x:si>
   <x:si>
     <x:t>7</x:t>
@@ -115,7 +118,7 @@
     <x:t>dungtdhe186461</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:23:14</x:t>
+    <x:t>11-12-2025 14:42:27</x:t>
   </x:si>
   <x:si>
     <x:t>8</x:t>
@@ -130,7 +133,7 @@
     <x:t>DuyCNHE187327</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:22:58</x:t>
+    <x:t>11-12-2025 14:42:10</x:t>
   </x:si>
   <x:si>
     <x:t>10</x:t>
@@ -139,6 +142,9 @@
     <x:t>duyldhe176352</x:t>
   </x:si>
   <x:si>
+    <x:t>11-12-2025 14:42:17</x:t>
+  </x:si>
+  <x:si>
     <x:t>11</x:t>
   </x:si>
   <x:si>
@@ -157,7 +163,7 @@
     <x:t>hieunqhe171297</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:23:16</x:t>
+    <x:t>11-12-2025 14:42:23</x:t>
   </x:si>
   <x:si>
     <x:t>14</x:t>
@@ -166,7 +172,7 @@
     <x:t>HoangHHHE182296</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:20:54</x:t>
+    <x:t>11-12-2025 14:42:21</x:t>
   </x:si>
   <x:si>
     <x:t>15</x:t>
@@ -187,18 +193,15 @@
     <x:t>linhmndhe186854</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:20:53</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11-12-2025 14:23:00</x:t>
-  </x:si>
-  <x:si>
     <x:t>18</x:t>
   </x:si>
   <x:si>
     <x:t>linhndhe172819</x:t>
   </x:si>
   <x:si>
+    <x:t>11-12-2025 14:40:09</x:t>
+  </x:si>
+  <x:si>
     <x:t>19</x:t>
   </x:si>
   <x:si>
@@ -211,7 +214,7 @@
     <x:t>manhcdhe176818</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:22:57</x:t>
+    <x:t>11-12-2025 14:42:20</x:t>
   </x:si>
   <x:si>
     <x:t>21</x:t>
@@ -226,9 +229,6 @@
     <x:t>nguyendvhe176752</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:22:55</x:t>
-  </x:si>
-  <x:si>
     <x:t>23</x:t>
   </x:si>
   <x:si>
@@ -253,10 +253,7 @@
     <x:t>tungbdhe172875</x:t>
   </x:si>
   <x:si>
-    <x:t>11-12-2025 14:20:56</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11-12-2025 14:20:57</x:t>
+    <x:t>11-12-2025 14:40:10</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -735,18 +732,18 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G3" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H3" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8">
       <x:c r="A4" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
         <x:v>8</x:v>
@@ -761,18 +758,18 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G4" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H4" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:8">
       <x:c r="A5" s="2" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
         <x:v>8</x:v>
@@ -781,16 +778,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F5" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="G5" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H5" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:8">
@@ -798,7 +795,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
         <x:v>8</x:v>
@@ -807,13 +804,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
         <x:v>13</x:v>
@@ -821,10 +818,10 @@
     </x:row>
     <x:row r="7" spans="1:8">
       <x:c r="A7" s="2" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C7" s="2" t="s">
         <x:v>8</x:v>
@@ -839,18 +836,18 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G7" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H7" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:8">
       <x:c r="A8" s="2" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B8" s="2" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C8" s="2" t="s">
         <x:v>8</x:v>
@@ -859,24 +856,24 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E8" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F8" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="G8" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H8" s="2" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:8">
       <x:c r="A9" s="2" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B9" s="2" t="s">
-        <x:v>35</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C9" s="2" t="s">
         <x:v>8</x:v>
@@ -894,15 +891,15 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="H9" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:8">
       <x:c r="A10" s="2" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B10" s="2" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C10" s="2" t="s">
         <x:v>8</x:v>
@@ -917,18 +914,18 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G10" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H10" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:8">
       <x:c r="A11" s="2" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B11" s="2" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C11" s="2" t="s">
         <x:v>8</x:v>
@@ -946,15 +943,15 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="H11" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:8">
       <x:c r="A12" s="2" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C12" s="2" t="s">
         <x:v>8</x:v>
@@ -972,15 +969,15 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="H12" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:8">
       <x:c r="A13" s="3" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
         <x:v>8</x:v>
@@ -989,24 +986,24 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:8">
       <x:c r="A14" s="2" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B14" s="2" t="s">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C14" s="2" t="s">
         <x:v>8</x:v>
@@ -1015,7 +1012,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E14" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F14" s="2" t="s">
         <x:v>12</x:v>
@@ -1024,15 +1021,15 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="H14" s="2" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:8">
       <x:c r="A15" s="2" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B15" s="2" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C15" s="2" t="s">
         <x:v>8</x:v>
@@ -1041,24 +1038,24 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E15" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F15" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="G15" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H15" s="2" t="s">
-        <x:v>38</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:8">
       <x:c r="A16" s="3" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
         <x:v>8</x:v>
@@ -1067,10 +1064,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
         <x:v>13</x:v>
@@ -1081,10 +1078,10 @@
     </x:row>
     <x:row r="17" spans="1:8">
       <x:c r="A17" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B17" s="2" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C17" s="2" t="s">
         <x:v>8</x:v>
@@ -1102,15 +1099,15 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="H17" s="2" t="s">
-        <x:v>30</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:8">
       <x:c r="A18" s="2" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B18" s="2" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C18" s="2" t="s">
         <x:v>8</x:v>
@@ -1119,16 +1116,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E18" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F18" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="G18" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H18" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:8">
@@ -1145,50 +1142,50 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:8">
       <x:c r="A20" s="3" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B20" s="3" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C20" s="3" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D20" s="3" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E20" s="3" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F20" s="3" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G20" s="3" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B20" s="3" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="C20" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D20" s="3" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="E20" s="3" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F20" s="3" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="G20" s="3" t="s">
-        <x:v>57</x:v>
-      </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:8">
       <x:c r="A21" s="2" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B21" s="2" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C21" s="2" t="s">
         <x:v>8</x:v>
@@ -1203,18 +1200,18 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G21" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H21" s="2" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:8">
       <x:c r="A22" s="2" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B22" s="2" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C22" s="2" t="s">
         <x:v>8</x:v>
@@ -1229,18 +1226,18 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G22" s="2" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H22" s="2" t="s">
-        <x:v>58</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:8">
       <x:c r="A23" s="2" t="s">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B23" s="2" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C23" s="2" t="s">
         <x:v>8</x:v>
@@ -1255,10 +1252,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="G23" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H23" s="2" t="s">
-        <x:v>70</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:8">
@@ -1275,16 +1272,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E24" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F24" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="G24" s="2" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H24" s="2" t="s">
-        <x:v>25</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:8">
@@ -1301,16 +1298,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:8">
@@ -1327,16 +1324,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>50</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:8">
@@ -1353,16 +1350,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
         <x:v>79</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>